<commit_message>
Add data quality analysis
</commit_message>
<xml_diff>
--- a/docs/data_dictionary.xlsx
+++ b/docs/data_dictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VISHNU KASHYAP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Guvi\cart2insights\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94FCD90-7F75-4E64-A640-49394B7745B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67FBC890-562E-417A-B76F-C1A8E1222328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -429,7 +429,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -439,12 +439,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -461,17 +455,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -752,7 +745,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
@@ -796,7 +789,7 @@
       <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" t="s">
         <v>103</v>
       </c>
       <c r="F2" t="s">
@@ -817,7 +810,7 @@
       <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" t="s">
         <v>63</v>
       </c>
       <c r="F3" t="s">
@@ -834,10 +827,10 @@
       <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
         <v>64</v>
       </c>
       <c r="F4" t="s">
@@ -857,7 +850,7 @@
       <c r="D5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" t="s">
         <v>65</v>
       </c>
       <c r="F5" t="s">
@@ -877,7 +870,7 @@
       <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" t="s">
         <v>66</v>
       </c>
       <c r="F6" t="s">
@@ -894,10 +887,10 @@
       <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
         <v>104</v>
       </c>
       <c r="F7" t="s">
@@ -917,7 +910,7 @@
       <c r="D8" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" t="s">
         <v>105</v>
       </c>
       <c r="F8" t="s">
@@ -937,7 +930,7 @@
       <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" t="s">
         <v>106</v>
       </c>
       <c r="F9" t="s">
@@ -957,7 +950,7 @@
       <c r="D10" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" t="s">
         <v>67</v>
       </c>
       <c r="F10" t="s">
@@ -977,7 +970,7 @@
       <c r="D11" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" t="s">
         <v>68</v>
       </c>
       <c r="F11" t="s">
@@ -997,10 +990,10 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" t="s">
         <v>107</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1017,7 +1010,7 @@
       <c r="D13" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" t="s">
         <v>108</v>
       </c>
       <c r="F13" t="s">
@@ -1037,7 +1030,7 @@
       <c r="D14" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" t="s">
         <v>69</v>
       </c>
       <c r="F14" t="s">
@@ -1057,7 +1050,7 @@
       <c r="D15" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" t="s">
         <v>70</v>
       </c>
       <c r="F15" t="s">
@@ -1074,10 +1067,10 @@
       <c r="C16" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" t="s">
         <v>71</v>
       </c>
       <c r="F16" t="s">
@@ -1097,7 +1090,7 @@
       <c r="D17" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" t="s">
         <v>72</v>
       </c>
       <c r="F17" t="s">
@@ -1117,7 +1110,7 @@
       <c r="D18" t="s">
         <v>23</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" t="s">
         <v>73</v>
       </c>
       <c r="F18" t="s">
@@ -1137,7 +1130,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" t="s">
         <v>74</v>
       </c>
       <c r="F19" t="s">
@@ -1157,7 +1150,7 @@
       <c r="D20" t="s">
         <v>20</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" t="s">
         <v>109</v>
       </c>
       <c r="F20" t="s">
@@ -1177,7 +1170,7 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" t="s">
         <v>110</v>
       </c>
       <c r="F21" t="s">
@@ -1197,7 +1190,7 @@
       <c r="D22" t="s">
         <v>20</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" t="s">
         <v>75</v>
       </c>
       <c r="F22" t="s">
@@ -1217,7 +1210,7 @@
       <c r="D23" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" t="s">
         <v>76</v>
       </c>
       <c r="F23" t="s">
@@ -1237,7 +1230,7 @@
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" t="s">
         <v>77</v>
       </c>
       <c r="F24" t="s">
@@ -1257,7 +1250,7 @@
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" t="s">
         <v>78</v>
       </c>
       <c r="F25" t="s">
@@ -1277,7 +1270,7 @@
       <c r="D26" t="s">
         <v>20</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" t="s">
         <v>79</v>
       </c>
       <c r="F26" t="s">
@@ -1297,7 +1290,7 @@
       <c r="D27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" t="s">
         <v>111</v>
       </c>
       <c r="F27" t="s">
@@ -1317,7 +1310,7 @@
       <c r="D28" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" t="s">
         <v>112</v>
       </c>
       <c r="F28" t="s">
@@ -1334,10 +1327,10 @@
       <c r="C29" t="s">
         <v>19</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" t="s">
         <v>80</v>
       </c>
       <c r="F29" t="s">
@@ -1354,10 +1347,10 @@
       <c r="C30" t="s">
         <v>19</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" t="s">
         <v>81</v>
       </c>
       <c r="F30" t="s">
@@ -1377,7 +1370,7 @@
       <c r="D31" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" t="s">
         <v>82</v>
       </c>
       <c r="F31" t="s">
@@ -1397,7 +1390,7 @@
       <c r="D32" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" t="s">
         <v>83</v>
       </c>
       <c r="F32" t="s">
@@ -1417,7 +1410,7 @@
       <c r="D33" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="5" t="s">
+      <c r="E33" t="s">
         <v>84</v>
       </c>
       <c r="F33" t="s">
@@ -1434,10 +1427,10 @@
       <c r="C34" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E34" s="5" t="s">
+      <c r="E34" t="s">
         <v>85</v>
       </c>
       <c r="F34" t="s">
@@ -1454,10 +1447,10 @@
       <c r="C35" t="s">
         <v>19</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" t="s">
         <v>86</v>
       </c>
       <c r="F35" t="s">
@@ -1474,10 +1467,10 @@
       <c r="C36" t="s">
         <v>19</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="E36" t="s">
         <v>87</v>
       </c>
       <c r="F36" t="s">
@@ -1494,10 +1487,10 @@
       <c r="C37" t="s">
         <v>19</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" t="s">
         <v>88</v>
       </c>
       <c r="F37" t="s">
@@ -1514,10 +1507,10 @@
       <c r="C38" t="s">
         <v>19</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="E38" t="s">
         <v>89</v>
       </c>
       <c r="F38" t="s">
@@ -1537,7 +1530,7 @@
       <c r="D39" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" t="s">
         <v>90</v>
       </c>
       <c r="F39" t="s">
@@ -1557,7 +1550,7 @@
       <c r="D40" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" t="s">
         <v>113</v>
       </c>
       <c r="F40" t="s">
@@ -1568,7 +1561,7 @@
       <c r="A41" t="s">
         <v>11</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C41" t="s">
@@ -1577,7 +1570,7 @@
       <c r="D41" t="s">
         <v>23</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" t="s">
         <v>91</v>
       </c>
       <c r="F41" t="s">
@@ -1588,7 +1581,7 @@
       <c r="A42" t="s">
         <v>11</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C42" t="s">
@@ -1597,7 +1590,7 @@
       <c r="D42" t="s">
         <v>23</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" t="s">
         <v>92</v>
       </c>
       <c r="F42" t="s">
@@ -1617,7 +1610,7 @@
       <c r="D43" t="s">
         <v>23</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="E43" t="s">
         <v>93</v>
       </c>
       <c r="F43" t="s">
@@ -1637,7 +1630,7 @@
       <c r="D44" t="s">
         <v>23</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="E44" t="s">
         <v>94</v>
       </c>
       <c r="F44" t="s">
@@ -1657,7 +1650,7 @@
       <c r="D45" t="s">
         <v>23</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="E45" t="s">
         <v>95</v>
       </c>
       <c r="F45" t="s">
@@ -1677,7 +1670,7 @@
       <c r="D46" t="s">
         <v>23</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="E46" t="s">
         <v>96</v>
       </c>
       <c r="F46" t="s">
@@ -1697,7 +1690,7 @@
       <c r="D47" t="s">
         <v>23</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="E47" t="s">
         <v>97</v>
       </c>
       <c r="F47" t="s">
@@ -1717,7 +1710,7 @@
       <c r="D48" t="s">
         <v>19</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="E48" t="s">
         <v>98</v>
       </c>
       <c r="F48" t="s">
@@ -1734,13 +1727,13 @@
       <c r="C49" t="s">
         <v>20</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E49" s="5" t="s">
+      <c r="D49" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E49" t="s">
         <v>99</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1757,7 +1750,7 @@
       <c r="D50" t="s">
         <v>19</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="E50" t="s">
         <v>100</v>
       </c>
       <c r="F50" t="s">
@@ -1777,7 +1770,7 @@
       <c r="D51" t="s">
         <v>19</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="E51" t="s">
         <v>101</v>
       </c>
       <c r="F51" t="s">
@@ -1797,7 +1790,7 @@
       <c r="D52" t="s">
         <v>19</v>
       </c>
-      <c r="E52" s="5" t="s">
+      <c r="E52" t="s">
         <v>114</v>
       </c>
       <c r="F52" t="s">
@@ -1817,12 +1810,15 @@
       <c r="D53" t="s">
         <v>19</v>
       </c>
-      <c r="E53" s="5" t="s">
+      <c r="E53" t="s">
         <v>102</v>
       </c>
       <c r="F53" t="s">
         <v>117</v>
       </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F55" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F53" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>